<commit_message>
Append and fill workbook columns for all available offset runs
</commit_message>
<xml_diff>
--- a/analysis/20261019-time-offset-xlsx/time_offset.xlsx
+++ b/analysis/20261019-time-offset-xlsx/time_offset.xlsx
@@ -410,13 +410,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E80"/>
+  <dimension ref="A1:Q80"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="27" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -432,8 +432,68 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>time offset 6024</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>time offset 6028</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>time offset 6035</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>time offset 6041</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>time offset 6045</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>time offset 6050</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>time offset 6054</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>time offset 6061</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>time offset 6065</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>time offset 6071</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>time offset 6075</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>time offset 6078</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -449,8 +509,44 @@
       <c r="E2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F2" s="1">
+        <v>0</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0</v>
+      </c>
+      <c r="I2" s="1">
+        <v>0</v>
+      </c>
+      <c r="J2" s="1">
+        <v>0</v>
+      </c>
+      <c r="K2" s="1">
+        <v>0</v>
+      </c>
+      <c r="L2" s="1">
+        <v>0</v>
+      </c>
+      <c r="M2" s="1">
+        <v>0</v>
+      </c>
+      <c r="N2" s="1">
+        <v>0</v>
+      </c>
+      <c r="O2" s="1">
+        <v>0</v>
+      </c>
+      <c r="P2" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>0</v>
       </c>
@@ -466,8 +562,44 @@
       <c r="E3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F3" s="1">
+        <v>0</v>
+      </c>
+      <c r="G3" s="1">
+        <v>0</v>
+      </c>
+      <c r="H3" s="1">
+        <v>0</v>
+      </c>
+      <c r="I3" s="1">
+        <v>0</v>
+      </c>
+      <c r="J3" s="1">
+        <v>0</v>
+      </c>
+      <c r="K3" s="1">
+        <v>0</v>
+      </c>
+      <c r="L3" s="1">
+        <v>0</v>
+      </c>
+      <c r="M3" s="1">
+        <v>0</v>
+      </c>
+      <c r="N3" s="1">
+        <v>0</v>
+      </c>
+      <c r="O3" s="1">
+        <v>0</v>
+      </c>
+      <c r="P3" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>0</v>
       </c>
@@ -483,8 +615,42 @@
       <c r="E4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F4" s="1">
+        <v>0</v>
+      </c>
+      <c r="G4" s="1">
+        <v>0</v>
+      </c>
+      <c r="H4" s="1">
+        <v>0</v>
+      </c>
+      <c r="I4" s="1">
+        <v>0</v>
+      </c>
+      <c r="J4" s="1">
+        <v>0</v>
+      </c>
+      <c r="K4" s="1">
+        <v>0</v>
+      </c>
+      <c r="L4" s="1">
+        <v>0</v>
+      </c>
+      <c r="M4" s="1">
+        <v>0</v>
+      </c>
+      <c r="N4" s="1">
+        <v>0</v>
+      </c>
+      <c r="O4" s="1">
+        <v>0</v>
+      </c>
+      <c r="P4" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="1"/>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>0</v>
       </c>
@@ -500,8 +666,44 @@
       <c r="E5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F5" s="1">
+        <v>0</v>
+      </c>
+      <c r="G5" s="1">
+        <v>0</v>
+      </c>
+      <c r="H5" s="1">
+        <v>0</v>
+      </c>
+      <c r="I5" s="1">
+        <v>0</v>
+      </c>
+      <c r="J5" s="1">
+        <v>0</v>
+      </c>
+      <c r="K5" s="1">
+        <v>0</v>
+      </c>
+      <c r="L5" s="1">
+        <v>0</v>
+      </c>
+      <c r="M5" s="1">
+        <v>0</v>
+      </c>
+      <c r="N5" s="1">
+        <v>0</v>
+      </c>
+      <c r="O5" s="1">
+        <v>0</v>
+      </c>
+      <c r="P5" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>0</v>
       </c>
@@ -517,8 +719,44 @@
       <c r="E6">
         <v>80</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F6" s="1">
+        <v>88</v>
+      </c>
+      <c r="G6" s="1">
+        <v>88</v>
+      </c>
+      <c r="H6" s="1">
+        <v>88</v>
+      </c>
+      <c r="I6" s="1">
+        <v>80</v>
+      </c>
+      <c r="J6" s="1">
+        <v>80</v>
+      </c>
+      <c r="K6" s="1">
+        <v>88</v>
+      </c>
+      <c r="L6" s="1">
+        <v>80</v>
+      </c>
+      <c r="M6" s="1">
+        <v>88</v>
+      </c>
+      <c r="N6" s="1">
+        <v>88</v>
+      </c>
+      <c r="O6" s="1">
+        <v>88</v>
+      </c>
+      <c r="P6" s="1">
+        <v>88</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>0</v>
       </c>
@@ -534,8 +772,44 @@
       <c r="E7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F7" s="1">
+        <v>0</v>
+      </c>
+      <c r="G7" s="1">
+        <v>0</v>
+      </c>
+      <c r="H7" s="1">
+        <v>0</v>
+      </c>
+      <c r="I7" s="1">
+        <v>0</v>
+      </c>
+      <c r="J7" s="1">
+        <v>0</v>
+      </c>
+      <c r="K7" s="1">
+        <v>0</v>
+      </c>
+      <c r="L7" s="1">
+        <v>0</v>
+      </c>
+      <c r="M7" s="1">
+        <v>0</v>
+      </c>
+      <c r="N7" s="1">
+        <v>0</v>
+      </c>
+      <c r="O7" s="1">
+        <v>0</v>
+      </c>
+      <c r="P7" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>0</v>
       </c>
@@ -551,8 +825,44 @@
       <c r="E8">
         <v>56</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F8" s="1">
+        <v>64</v>
+      </c>
+      <c r="G8" s="1">
+        <v>64</v>
+      </c>
+      <c r="H8" s="1">
+        <v>64</v>
+      </c>
+      <c r="I8" s="1">
+        <v>64</v>
+      </c>
+      <c r="J8" s="1">
+        <v>64</v>
+      </c>
+      <c r="K8" s="1">
+        <v>64</v>
+      </c>
+      <c r="L8" s="1">
+        <v>64</v>
+      </c>
+      <c r="M8" s="1">
+        <v>64</v>
+      </c>
+      <c r="N8" s="1">
+        <v>64</v>
+      </c>
+      <c r="O8" s="1">
+        <v>64</v>
+      </c>
+      <c r="P8" s="1">
+        <v>64</v>
+      </c>
+      <c r="Q8" s="1">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>0</v>
       </c>
@@ -568,8 +878,44 @@
       <c r="E9">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F9" s="1">
+        <v>0</v>
+      </c>
+      <c r="G9" s="1">
+        <v>0</v>
+      </c>
+      <c r="H9" s="1">
+        <v>0</v>
+      </c>
+      <c r="I9" s="1">
+        <v>0</v>
+      </c>
+      <c r="J9" s="1">
+        <v>0</v>
+      </c>
+      <c r="K9" s="1">
+        <v>0</v>
+      </c>
+      <c r="L9" s="1">
+        <v>0</v>
+      </c>
+      <c r="M9" s="1">
+        <v>0</v>
+      </c>
+      <c r="N9" s="1">
+        <v>0</v>
+      </c>
+      <c r="O9" s="1">
+        <v>0</v>
+      </c>
+      <c r="P9" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>0</v>
       </c>
@@ -585,8 +931,44 @@
       <c r="E10">
         <v>-0</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F10" s="1">
+        <v>0</v>
+      </c>
+      <c r="G10" s="1">
+        <v>0</v>
+      </c>
+      <c r="H10" s="1">
+        <v>0</v>
+      </c>
+      <c r="I10" s="1">
+        <v>0</v>
+      </c>
+      <c r="J10" s="1">
+        <v>-0</v>
+      </c>
+      <c r="K10" s="1">
+        <v>0</v>
+      </c>
+      <c r="L10" s="1">
+        <v>0</v>
+      </c>
+      <c r="M10" s="1">
+        <v>-0</v>
+      </c>
+      <c r="N10" s="1">
+        <v>0</v>
+      </c>
+      <c r="O10" s="1">
+        <v>0</v>
+      </c>
+      <c r="P10" s="1">
+        <v>-0</v>
+      </c>
+      <c r="Q10" s="1">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>0</v>
       </c>
@@ -602,8 +984,44 @@
       <c r="E11">
         <v>16</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F11" s="1">
+        <v>16</v>
+      </c>
+      <c r="G11" s="1">
+        <v>16</v>
+      </c>
+      <c r="H11" s="1">
+        <v>24</v>
+      </c>
+      <c r="I11" s="1">
+        <v>24</v>
+      </c>
+      <c r="J11" s="1">
+        <v>16</v>
+      </c>
+      <c r="K11" s="1">
+        <v>16</v>
+      </c>
+      <c r="L11" s="1">
+        <v>16</v>
+      </c>
+      <c r="M11" s="1">
+        <v>8</v>
+      </c>
+      <c r="N11" s="1">
+        <v>8</v>
+      </c>
+      <c r="O11" s="1">
+        <v>16</v>
+      </c>
+      <c r="P11" s="1">
+        <v>16</v>
+      </c>
+      <c r="Q11" s="1">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>0</v>
       </c>
@@ -619,8 +1037,44 @@
       <c r="E12">
         <v>8</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F12" s="1">
+        <v>8</v>
+      </c>
+      <c r="G12" s="1">
+        <v>8</v>
+      </c>
+      <c r="H12" s="1">
+        <v>8</v>
+      </c>
+      <c r="I12" s="1">
+        <v>8</v>
+      </c>
+      <c r="J12" s="1">
+        <v>8</v>
+      </c>
+      <c r="K12" s="1">
+        <v>8</v>
+      </c>
+      <c r="L12" s="1">
+        <v>0</v>
+      </c>
+      <c r="M12" s="1">
+        <v>0</v>
+      </c>
+      <c r="N12" s="1">
+        <v>0</v>
+      </c>
+      <c r="O12" s="1">
+        <v>8</v>
+      </c>
+      <c r="P12" s="1">
+        <v>8</v>
+      </c>
+      <c r="Q12" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>0</v>
       </c>
@@ -636,8 +1090,44 @@
       <c r="E13">
         <v>80</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F13" s="1">
+        <v>88</v>
+      </c>
+      <c r="G13" s="1">
+        <v>80</v>
+      </c>
+      <c r="H13" s="1">
+        <v>88</v>
+      </c>
+      <c r="I13" s="1">
+        <v>96</v>
+      </c>
+      <c r="J13" s="1">
+        <v>80</v>
+      </c>
+      <c r="K13" s="1">
+        <v>80</v>
+      </c>
+      <c r="L13" s="1">
+        <v>80</v>
+      </c>
+      <c r="M13" s="1">
+        <v>80</v>
+      </c>
+      <c r="N13" s="1">
+        <v>80</v>
+      </c>
+      <c r="O13" s="1">
+        <v>80</v>
+      </c>
+      <c r="P13" s="1">
+        <v>88</v>
+      </c>
+      <c r="Q13" s="1">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>0</v>
       </c>
@@ -653,8 +1143,44 @@
       <c r="E14">
         <v>56</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F14" s="1">
+        <v>64</v>
+      </c>
+      <c r="G14" s="1">
+        <v>64</v>
+      </c>
+      <c r="H14" s="1">
+        <v>72</v>
+      </c>
+      <c r="I14" s="1">
+        <v>72</v>
+      </c>
+      <c r="J14" s="1">
+        <v>56</v>
+      </c>
+      <c r="K14" s="1">
+        <v>64</v>
+      </c>
+      <c r="L14" s="1">
+        <v>56</v>
+      </c>
+      <c r="M14" s="1">
+        <v>56</v>
+      </c>
+      <c r="N14" s="1">
+        <v>56</v>
+      </c>
+      <c r="O14" s="1">
+        <v>56</v>
+      </c>
+      <c r="P14" s="1">
+        <v>56</v>
+      </c>
+      <c r="Q14" s="1">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>0</v>
       </c>
@@ -670,8 +1196,44 @@
       <c r="E15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F15" s="1">
+        <v>0</v>
+      </c>
+      <c r="G15" s="1">
+        <v>0</v>
+      </c>
+      <c r="H15" s="1">
+        <v>0</v>
+      </c>
+      <c r="I15" s="1">
+        <v>0</v>
+      </c>
+      <c r="J15" s="1">
+        <v>0</v>
+      </c>
+      <c r="K15" s="1">
+        <v>0</v>
+      </c>
+      <c r="L15" s="1">
+        <v>0</v>
+      </c>
+      <c r="M15" s="1">
+        <v>0</v>
+      </c>
+      <c r="N15" s="1">
+        <v>0</v>
+      </c>
+      <c r="O15" s="1">
+        <v>0</v>
+      </c>
+      <c r="P15" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>0</v>
       </c>
@@ -687,8 +1249,44 @@
       <c r="E16">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F16" s="1">
+        <v>0</v>
+      </c>
+      <c r="G16" s="1">
+        <v>0</v>
+      </c>
+      <c r="H16" s="1">
+        <v>0</v>
+      </c>
+      <c r="I16" s="1">
+        <v>0</v>
+      </c>
+      <c r="J16" s="1">
+        <v>0</v>
+      </c>
+      <c r="K16" s="1">
+        <v>0</v>
+      </c>
+      <c r="L16" s="1">
+        <v>0</v>
+      </c>
+      <c r="M16" s="1">
+        <v>0</v>
+      </c>
+      <c r="N16" s="1">
+        <v>0</v>
+      </c>
+      <c r="O16" s="1">
+        <v>0</v>
+      </c>
+      <c r="P16" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>0</v>
       </c>
@@ -704,8 +1302,44 @@
       <c r="E17">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F17" s="1">
+        <v>0</v>
+      </c>
+      <c r="G17" s="1">
+        <v>0</v>
+      </c>
+      <c r="H17" s="1">
+        <v>0</v>
+      </c>
+      <c r="I17" s="1">
+        <v>0</v>
+      </c>
+      <c r="J17" s="1">
+        <v>0</v>
+      </c>
+      <c r="K17" s="1">
+        <v>0</v>
+      </c>
+      <c r="L17" s="1">
+        <v>0</v>
+      </c>
+      <c r="M17" s="1">
+        <v>0</v>
+      </c>
+      <c r="N17" s="1">
+        <v>0</v>
+      </c>
+      <c r="O17" s="1">
+        <v>0</v>
+      </c>
+      <c r="P17" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>0</v>
       </c>
@@ -721,8 +1355,44 @@
       <c r="E18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F18" s="1">
+        <v>0</v>
+      </c>
+      <c r="G18" s="1">
+        <v>0</v>
+      </c>
+      <c r="H18" s="1">
+        <v>0</v>
+      </c>
+      <c r="I18" s="1">
+        <v>0</v>
+      </c>
+      <c r="J18" s="1">
+        <v>0</v>
+      </c>
+      <c r="K18" s="1">
+        <v>0</v>
+      </c>
+      <c r="L18" s="1">
+        <v>0</v>
+      </c>
+      <c r="M18" s="1">
+        <v>0</v>
+      </c>
+      <c r="N18" s="1">
+        <v>0</v>
+      </c>
+      <c r="O18" s="1">
+        <v>0</v>
+      </c>
+      <c r="P18" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>0</v>
       </c>
@@ -738,8 +1408,44 @@
       <c r="E19">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F19" s="1">
+        <v>0</v>
+      </c>
+      <c r="G19" s="1">
+        <v>0</v>
+      </c>
+      <c r="H19" s="1">
+        <v>0</v>
+      </c>
+      <c r="I19" s="1">
+        <v>0</v>
+      </c>
+      <c r="J19" s="1">
+        <v>0</v>
+      </c>
+      <c r="K19" s="1">
+        <v>0</v>
+      </c>
+      <c r="L19" s="1">
+        <v>0</v>
+      </c>
+      <c r="M19" s="1">
+        <v>0</v>
+      </c>
+      <c r="N19" s="1">
+        <v>0</v>
+      </c>
+      <c r="O19" s="1">
+        <v>0</v>
+      </c>
+      <c r="P19" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>0</v>
       </c>
@@ -755,8 +1461,44 @@
       <c r="E20">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F20" s="1">
+        <v>0</v>
+      </c>
+      <c r="G20" s="1">
+        <v>0</v>
+      </c>
+      <c r="H20" s="1">
+        <v>0</v>
+      </c>
+      <c r="I20" s="1">
+        <v>0</v>
+      </c>
+      <c r="J20" s="1">
+        <v>0</v>
+      </c>
+      <c r="K20" s="1">
+        <v>0</v>
+      </c>
+      <c r="L20" s="1">
+        <v>0</v>
+      </c>
+      <c r="M20" s="1">
+        <v>0</v>
+      </c>
+      <c r="N20" s="1">
+        <v>0</v>
+      </c>
+      <c r="O20" s="1">
+        <v>0</v>
+      </c>
+      <c r="P20" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>0</v>
       </c>
@@ -772,8 +1514,44 @@
       <c r="E21">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F21" s="1">
+        <v>0</v>
+      </c>
+      <c r="G21" s="1">
+        <v>0</v>
+      </c>
+      <c r="H21" s="1">
+        <v>0</v>
+      </c>
+      <c r="I21" s="1">
+        <v>0</v>
+      </c>
+      <c r="J21" s="1">
+        <v>0</v>
+      </c>
+      <c r="K21" s="1">
+        <v>0</v>
+      </c>
+      <c r="L21" s="1">
+        <v>0</v>
+      </c>
+      <c r="M21" s="1">
+        <v>0</v>
+      </c>
+      <c r="N21" s="1">
+        <v>0</v>
+      </c>
+      <c r="O21" s="1">
+        <v>0</v>
+      </c>
+      <c r="P21" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>0</v>
       </c>
@@ -789,8 +1567,44 @@
       <c r="E22">
         <v>-0</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F22" s="1">
+        <v>0</v>
+      </c>
+      <c r="G22" s="1">
+        <v>8</v>
+      </c>
+      <c r="H22" s="1">
+        <v>8</v>
+      </c>
+      <c r="I22" s="1">
+        <v>8</v>
+      </c>
+      <c r="J22" s="1">
+        <v>8</v>
+      </c>
+      <c r="K22" s="1">
+        <v>8</v>
+      </c>
+      <c r="L22" s="1">
+        <v>0</v>
+      </c>
+      <c r="M22" s="1">
+        <v>0</v>
+      </c>
+      <c r="N22" s="1">
+        <v>0</v>
+      </c>
+      <c r="O22" s="1">
+        <v>0</v>
+      </c>
+      <c r="P22" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>0</v>
       </c>
@@ -806,8 +1620,44 @@
       <c r="E23">
         <v>56</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F23" s="1">
+        <v>56</v>
+      </c>
+      <c r="G23" s="1">
+        <v>56</v>
+      </c>
+      <c r="H23" s="1">
+        <v>56</v>
+      </c>
+      <c r="I23" s="1">
+        <v>56</v>
+      </c>
+      <c r="J23" s="1">
+        <v>56</v>
+      </c>
+      <c r="K23" s="1">
+        <v>64</v>
+      </c>
+      <c r="L23" s="1">
+        <v>48</v>
+      </c>
+      <c r="M23" s="1">
+        <v>48</v>
+      </c>
+      <c r="N23" s="1">
+        <v>48</v>
+      </c>
+      <c r="O23" s="1">
+        <v>48</v>
+      </c>
+      <c r="P23" s="1">
+        <v>56</v>
+      </c>
+      <c r="Q23" s="1">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>0</v>
       </c>
@@ -823,8 +1673,42 @@
       <c r="E24">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F24" s="1">
+        <v>0</v>
+      </c>
+      <c r="G24" s="1">
+        <v>-0</v>
+      </c>
+      <c r="H24" s="1">
+        <v>0</v>
+      </c>
+      <c r="I24" s="1">
+        <v>0</v>
+      </c>
+      <c r="J24" s="1">
+        <v>-0</v>
+      </c>
+      <c r="K24" s="1">
+        <v>0</v>
+      </c>
+      <c r="L24" s="1">
+        <v>-0</v>
+      </c>
+      <c r="M24" s="1">
+        <v>0</v>
+      </c>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1">
+        <v>0</v>
+      </c>
+      <c r="P24" s="1">
+        <v>-0</v>
+      </c>
+      <c r="Q24" s="1">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>0</v>
       </c>
@@ -840,8 +1724,44 @@
       <c r="E25">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F25" s="1">
+        <v>0</v>
+      </c>
+      <c r="G25" s="1">
+        <v>0</v>
+      </c>
+      <c r="H25" s="1">
+        <v>0</v>
+      </c>
+      <c r="I25" s="1">
+        <v>0</v>
+      </c>
+      <c r="J25" s="1">
+        <v>0</v>
+      </c>
+      <c r="K25" s="1">
+        <v>0</v>
+      </c>
+      <c r="L25" s="1">
+        <v>0</v>
+      </c>
+      <c r="M25" s="1">
+        <v>0</v>
+      </c>
+      <c r="N25" s="1">
+        <v>0</v>
+      </c>
+      <c r="O25" s="1">
+        <v>0</v>
+      </c>
+      <c r="P25" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>0</v>
       </c>
@@ -857,8 +1777,44 @@
       <c r="E26">
         <v>32</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F26" s="1">
+        <v>40</v>
+      </c>
+      <c r="G26" s="1">
+        <v>40</v>
+      </c>
+      <c r="H26" s="1">
+        <v>32</v>
+      </c>
+      <c r="I26" s="1">
+        <v>48</v>
+      </c>
+      <c r="J26" s="1">
+        <v>40</v>
+      </c>
+      <c r="K26" s="1">
+        <v>40</v>
+      </c>
+      <c r="L26" s="1">
+        <v>32</v>
+      </c>
+      <c r="M26" s="1">
+        <v>32</v>
+      </c>
+      <c r="N26" s="1">
+        <v>32</v>
+      </c>
+      <c r="O26" s="1">
+        <v>32</v>
+      </c>
+      <c r="P26" s="1">
+        <v>32</v>
+      </c>
+      <c r="Q26" s="1">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>0</v>
       </c>
@@ -874,8 +1830,44 @@
       <c r="E27">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F27" s="1">
+        <v>0</v>
+      </c>
+      <c r="G27" s="1">
+        <v>0</v>
+      </c>
+      <c r="H27" s="1">
+        <v>0</v>
+      </c>
+      <c r="I27" s="1">
+        <v>0</v>
+      </c>
+      <c r="J27" s="1">
+        <v>0</v>
+      </c>
+      <c r="K27" s="1">
+        <v>0</v>
+      </c>
+      <c r="L27" s="1">
+        <v>0</v>
+      </c>
+      <c r="M27" s="1">
+        <v>0</v>
+      </c>
+      <c r="N27" s="1">
+        <v>0</v>
+      </c>
+      <c r="O27" s="1">
+        <v>0</v>
+      </c>
+      <c r="P27" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>0</v>
       </c>
@@ -891,8 +1883,44 @@
       <c r="E28">
         <v>-8</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F28" s="1">
+        <v>-8</v>
+      </c>
+      <c r="G28" s="1">
+        <v>-0</v>
+      </c>
+      <c r="H28" s="1">
+        <v>-0</v>
+      </c>
+      <c r="I28" s="1">
+        <v>-8</v>
+      </c>
+      <c r="J28" s="1">
+        <v>-8</v>
+      </c>
+      <c r="K28" s="1">
+        <v>-0</v>
+      </c>
+      <c r="L28" s="1">
+        <v>-8</v>
+      </c>
+      <c r="M28" s="1">
+        <v>-8</v>
+      </c>
+      <c r="N28" s="1">
+        <v>-8</v>
+      </c>
+      <c r="O28" s="1">
+        <v>-0</v>
+      </c>
+      <c r="P28" s="1">
+        <v>-0</v>
+      </c>
+      <c r="Q28" s="1">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>0</v>
       </c>
@@ -908,8 +1936,44 @@
       <c r="E29">
         <v>56</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F29" s="1">
+        <v>56</v>
+      </c>
+      <c r="G29" s="1">
+        <v>64</v>
+      </c>
+      <c r="H29" s="1">
+        <v>56</v>
+      </c>
+      <c r="I29" s="1">
+        <v>64</v>
+      </c>
+      <c r="J29" s="1">
+        <v>56</v>
+      </c>
+      <c r="K29" s="1">
+        <v>64</v>
+      </c>
+      <c r="L29" s="1">
+        <v>56</v>
+      </c>
+      <c r="M29" s="1">
+        <v>48</v>
+      </c>
+      <c r="N29" s="1">
+        <v>56</v>
+      </c>
+      <c r="O29" s="1">
+        <v>56</v>
+      </c>
+      <c r="P29" s="1">
+        <v>56</v>
+      </c>
+      <c r="Q29" s="1">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>0</v>
       </c>
@@ -925,8 +1989,44 @@
       <c r="E30">
         <v>0</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F30" s="1">
+        <v>0</v>
+      </c>
+      <c r="G30" s="1">
+        <v>0</v>
+      </c>
+      <c r="H30" s="1">
+        <v>0</v>
+      </c>
+      <c r="I30" s="1">
+        <v>0</v>
+      </c>
+      <c r="J30" s="1">
+        <v>0</v>
+      </c>
+      <c r="K30" s="1">
+        <v>0</v>
+      </c>
+      <c r="L30" s="1">
+        <v>0</v>
+      </c>
+      <c r="M30" s="1">
+        <v>0</v>
+      </c>
+      <c r="N30" s="1">
+        <v>0</v>
+      </c>
+      <c r="O30" s="1">
+        <v>0</v>
+      </c>
+      <c r="P30" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>0</v>
       </c>
@@ -942,8 +2042,44 @@
       <c r="E31">
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F31" s="1">
+        <v>0</v>
+      </c>
+      <c r="G31" s="1">
+        <v>0</v>
+      </c>
+      <c r="H31" s="1">
+        <v>0</v>
+      </c>
+      <c r="I31" s="1">
+        <v>0</v>
+      </c>
+      <c r="J31" s="1">
+        <v>0</v>
+      </c>
+      <c r="K31" s="1">
+        <v>0</v>
+      </c>
+      <c r="L31" s="1">
+        <v>0</v>
+      </c>
+      <c r="M31" s="1">
+        <v>0</v>
+      </c>
+      <c r="N31" s="1">
+        <v>0</v>
+      </c>
+      <c r="O31" s="1">
+        <v>0</v>
+      </c>
+      <c r="P31" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>0</v>
       </c>
@@ -959,8 +2095,44 @@
       <c r="E32">
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F32" s="1">
+        <v>0</v>
+      </c>
+      <c r="G32" s="1">
+        <v>0</v>
+      </c>
+      <c r="H32" s="1">
+        <v>0</v>
+      </c>
+      <c r="I32" s="1">
+        <v>0</v>
+      </c>
+      <c r="J32" s="1">
+        <v>0</v>
+      </c>
+      <c r="K32" s="1">
+        <v>0</v>
+      </c>
+      <c r="L32" s="1">
+        <v>0</v>
+      </c>
+      <c r="M32" s="1">
+        <v>0</v>
+      </c>
+      <c r="N32" s="1">
+        <v>0</v>
+      </c>
+      <c r="O32" s="1">
+        <v>0</v>
+      </c>
+      <c r="P32" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>0</v>
       </c>
@@ -976,8 +2148,44 @@
       <c r="E33">
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F33" s="1">
+        <v>0</v>
+      </c>
+      <c r="G33" s="1">
+        <v>0</v>
+      </c>
+      <c r="H33" s="1">
+        <v>0</v>
+      </c>
+      <c r="I33" s="1">
+        <v>0</v>
+      </c>
+      <c r="J33" s="1">
+        <v>0</v>
+      </c>
+      <c r="K33" s="1">
+        <v>0</v>
+      </c>
+      <c r="L33" s="1">
+        <v>0</v>
+      </c>
+      <c r="M33" s="1">
+        <v>0</v>
+      </c>
+      <c r="N33" s="1">
+        <v>0</v>
+      </c>
+      <c r="O33" s="1">
+        <v>0</v>
+      </c>
+      <c r="P33" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>0</v>
       </c>
@@ -993,8 +2201,44 @@
       <c r="E34">
         <v>40</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F34" s="1">
+        <v>40</v>
+      </c>
+      <c r="G34" s="1">
+        <v>40</v>
+      </c>
+      <c r="H34" s="1">
+        <v>40</v>
+      </c>
+      <c r="I34" s="1">
+        <v>40</v>
+      </c>
+      <c r="J34" s="1">
+        <v>40</v>
+      </c>
+      <c r="K34" s="1">
+        <v>40</v>
+      </c>
+      <c r="L34" s="1">
+        <v>32</v>
+      </c>
+      <c r="M34" s="1">
+        <v>40</v>
+      </c>
+      <c r="N34" s="1">
+        <v>40</v>
+      </c>
+      <c r="O34" s="1">
+        <v>40</v>
+      </c>
+      <c r="P34" s="1">
+        <v>40</v>
+      </c>
+      <c r="Q34" s="1">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>0</v>
       </c>
@@ -1010,8 +2254,44 @@
       <c r="E35">
         <v>32</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F35" s="1">
+        <v>40</v>
+      </c>
+      <c r="G35" s="1">
+        <v>32</v>
+      </c>
+      <c r="H35" s="1">
+        <v>40</v>
+      </c>
+      <c r="I35" s="1">
+        <v>40</v>
+      </c>
+      <c r="J35" s="1">
+        <v>32</v>
+      </c>
+      <c r="K35" s="1">
+        <v>40</v>
+      </c>
+      <c r="L35" s="1">
+        <v>40</v>
+      </c>
+      <c r="M35" s="1">
+        <v>24</v>
+      </c>
+      <c r="N35" s="1">
+        <v>32</v>
+      </c>
+      <c r="O35" s="1">
+        <v>32</v>
+      </c>
+      <c r="P35" s="1">
+        <v>40</v>
+      </c>
+      <c r="Q35" s="1">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>0</v>
       </c>
@@ -1027,8 +2307,44 @@
       <c r="E36">
         <v>32</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F36" s="1">
+        <v>40</v>
+      </c>
+      <c r="G36" s="1">
+        <v>40</v>
+      </c>
+      <c r="H36" s="1">
+        <v>40</v>
+      </c>
+      <c r="I36" s="1">
+        <v>40</v>
+      </c>
+      <c r="J36" s="1">
+        <v>32</v>
+      </c>
+      <c r="K36" s="1">
+        <v>40</v>
+      </c>
+      <c r="L36" s="1">
+        <v>40</v>
+      </c>
+      <c r="M36" s="1">
+        <v>32</v>
+      </c>
+      <c r="N36" s="1">
+        <v>40</v>
+      </c>
+      <c r="O36" s="1">
+        <v>40</v>
+      </c>
+      <c r="P36" s="1">
+        <v>40</v>
+      </c>
+      <c r="Q36" s="1">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>0</v>
       </c>
@@ -1044,8 +2360,44 @@
       <c r="E37">
         <v>40</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F37" s="1">
+        <v>48</v>
+      </c>
+      <c r="G37" s="1">
+        <v>40</v>
+      </c>
+      <c r="H37" s="1">
+        <v>40</v>
+      </c>
+      <c r="I37" s="1">
+        <v>40</v>
+      </c>
+      <c r="J37" s="1">
+        <v>40</v>
+      </c>
+      <c r="K37" s="1">
+        <v>48</v>
+      </c>
+      <c r="L37" s="1">
+        <v>40</v>
+      </c>
+      <c r="M37" s="1">
+        <v>32</v>
+      </c>
+      <c r="N37" s="1">
+        <v>40</v>
+      </c>
+      <c r="O37" s="1">
+        <v>40</v>
+      </c>
+      <c r="P37" s="1">
+        <v>40</v>
+      </c>
+      <c r="Q37" s="1">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>0</v>
       </c>
@@ -1061,8 +2413,44 @@
       <c r="E38">
         <v>40</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F38" s="1">
+        <v>40</v>
+      </c>
+      <c r="G38" s="1">
+        <v>40</v>
+      </c>
+      <c r="H38" s="1">
+        <v>40</v>
+      </c>
+      <c r="I38" s="1">
+        <v>40</v>
+      </c>
+      <c r="J38" s="1">
+        <v>40</v>
+      </c>
+      <c r="K38" s="1">
+        <v>48</v>
+      </c>
+      <c r="L38" s="1">
+        <v>32</v>
+      </c>
+      <c r="M38" s="1">
+        <v>32</v>
+      </c>
+      <c r="N38" s="1">
+        <v>32</v>
+      </c>
+      <c r="O38" s="1">
+        <v>32</v>
+      </c>
+      <c r="P38" s="1">
+        <v>32</v>
+      </c>
+      <c r="Q38" s="1">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>0</v>
       </c>
@@ -1078,8 +2466,44 @@
       <c r="E39">
         <v>48</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F39" s="1">
+        <v>56</v>
+      </c>
+      <c r="G39" s="1">
+        <v>48</v>
+      </c>
+      <c r="H39" s="1">
+        <v>48</v>
+      </c>
+      <c r="I39" s="1">
+        <v>48</v>
+      </c>
+      <c r="J39" s="1">
+        <v>48</v>
+      </c>
+      <c r="K39" s="1">
+        <v>56</v>
+      </c>
+      <c r="L39" s="1">
+        <v>48</v>
+      </c>
+      <c r="M39" s="1">
+        <v>40</v>
+      </c>
+      <c r="N39" s="1">
+        <v>48</v>
+      </c>
+      <c r="O39" s="1">
+        <v>48</v>
+      </c>
+      <c r="P39" s="1">
+        <v>48</v>
+      </c>
+      <c r="Q39" s="1">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>0</v>
       </c>
@@ -1095,8 +2519,44 @@
       <c r="E40">
         <v>48</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F40" s="1">
+        <v>56</v>
+      </c>
+      <c r="G40" s="1">
+        <v>48</v>
+      </c>
+      <c r="H40" s="1">
+        <v>48</v>
+      </c>
+      <c r="I40" s="1">
+        <v>48</v>
+      </c>
+      <c r="J40" s="1">
+        <v>48</v>
+      </c>
+      <c r="K40" s="1">
+        <v>56</v>
+      </c>
+      <c r="L40" s="1">
+        <v>48</v>
+      </c>
+      <c r="M40" s="1">
+        <v>48</v>
+      </c>
+      <c r="N40" s="1">
+        <v>48</v>
+      </c>
+      <c r="O40" s="1">
+        <v>48</v>
+      </c>
+      <c r="P40" s="1">
+        <v>48</v>
+      </c>
+      <c r="Q40" s="1">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>0</v>
       </c>
@@ -1112,8 +2572,44 @@
       <c r="E41">
         <v>40</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F41" s="1">
+        <v>48</v>
+      </c>
+      <c r="G41" s="1">
+        <v>40</v>
+      </c>
+      <c r="H41" s="1">
+        <v>40</v>
+      </c>
+      <c r="I41" s="1">
+        <v>40</v>
+      </c>
+      <c r="J41" s="1">
+        <v>40</v>
+      </c>
+      <c r="K41" s="1">
+        <v>48</v>
+      </c>
+      <c r="L41" s="1">
+        <v>40</v>
+      </c>
+      <c r="M41" s="1">
+        <v>40</v>
+      </c>
+      <c r="N41" s="1">
+        <v>40</v>
+      </c>
+      <c r="O41" s="1">
+        <v>40</v>
+      </c>
+      <c r="P41" s="1">
+        <v>40</v>
+      </c>
+      <c r="Q41" s="1">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>0</v>
       </c>
@@ -1129,8 +2625,44 @@
       <c r="E42">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F42" s="1">
+        <v>0</v>
+      </c>
+      <c r="G42" s="1">
+        <v>0</v>
+      </c>
+      <c r="H42" s="1">
+        <v>0</v>
+      </c>
+      <c r="I42" s="1">
+        <v>0</v>
+      </c>
+      <c r="J42" s="1">
+        <v>0</v>
+      </c>
+      <c r="K42" s="1">
+        <v>0</v>
+      </c>
+      <c r="L42" s="1">
+        <v>0</v>
+      </c>
+      <c r="M42" s="1">
+        <v>0</v>
+      </c>
+      <c r="N42" s="1">
+        <v>0</v>
+      </c>
+      <c r="O42" s="1">
+        <v>0</v>
+      </c>
+      <c r="P42" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>0</v>
       </c>
@@ -1146,8 +2678,44 @@
       <c r="E43">
         <v>48</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F43" s="1">
+        <v>48</v>
+      </c>
+      <c r="G43" s="1">
+        <v>48</v>
+      </c>
+      <c r="H43" s="1">
+        <v>48</v>
+      </c>
+      <c r="I43" s="1">
+        <v>56</v>
+      </c>
+      <c r="J43" s="1">
+        <v>48</v>
+      </c>
+      <c r="K43" s="1">
+        <v>48</v>
+      </c>
+      <c r="L43" s="1">
+        <v>40</v>
+      </c>
+      <c r="M43" s="1">
+        <v>40</v>
+      </c>
+      <c r="N43" s="1">
+        <v>40</v>
+      </c>
+      <c r="O43" s="1">
+        <v>40</v>
+      </c>
+      <c r="P43" s="1">
+        <v>48</v>
+      </c>
+      <c r="Q43" s="1">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>0</v>
       </c>
@@ -1163,8 +2731,44 @@
       <c r="E44">
         <v>48</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F44" s="1">
+        <v>56</v>
+      </c>
+      <c r="G44" s="1">
+        <v>56</v>
+      </c>
+      <c r="H44" s="1">
+        <v>56</v>
+      </c>
+      <c r="I44" s="1">
+        <v>56</v>
+      </c>
+      <c r="J44" s="1">
+        <v>48</v>
+      </c>
+      <c r="K44" s="1">
+        <v>48</v>
+      </c>
+      <c r="L44" s="1">
+        <v>48</v>
+      </c>
+      <c r="M44" s="1">
+        <v>40</v>
+      </c>
+      <c r="N44" s="1">
+        <v>48</v>
+      </c>
+      <c r="O44" s="1">
+        <v>48</v>
+      </c>
+      <c r="P44" s="1">
+        <v>48</v>
+      </c>
+      <c r="Q44" s="1">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>0</v>
       </c>
@@ -1180,8 +2784,44 @@
       <c r="E45">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F45" s="1">
+        <v>0</v>
+      </c>
+      <c r="G45" s="1">
+        <v>0</v>
+      </c>
+      <c r="H45" s="1">
+        <v>0</v>
+      </c>
+      <c r="I45" s="1">
+        <v>0</v>
+      </c>
+      <c r="J45" s="1">
+        <v>24</v>
+      </c>
+      <c r="K45" s="1">
+        <v>32</v>
+      </c>
+      <c r="L45" s="1">
+        <v>32</v>
+      </c>
+      <c r="M45" s="1">
+        <v>24</v>
+      </c>
+      <c r="N45" s="1">
+        <v>24</v>
+      </c>
+      <c r="O45" s="1">
+        <v>24</v>
+      </c>
+      <c r="P45" s="1">
+        <v>32</v>
+      </c>
+      <c r="Q45" s="1">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>0</v>
       </c>
@@ -1197,8 +2837,44 @@
       <c r="E46">
         <v>0</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F46" s="1">
+        <v>0</v>
+      </c>
+      <c r="G46" s="1">
+        <v>0</v>
+      </c>
+      <c r="H46" s="1">
+        <v>0</v>
+      </c>
+      <c r="I46" s="1">
+        <v>0</v>
+      </c>
+      <c r="J46" s="1">
+        <v>0</v>
+      </c>
+      <c r="K46" s="1">
+        <v>0</v>
+      </c>
+      <c r="L46" s="1">
+        <v>0</v>
+      </c>
+      <c r="M46" s="1">
+        <v>0</v>
+      </c>
+      <c r="N46" s="1">
+        <v>0</v>
+      </c>
+      <c r="O46" s="1">
+        <v>0</v>
+      </c>
+      <c r="P46" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q46" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>0</v>
       </c>
@@ -1214,8 +2890,44 @@
       <c r="E47">
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F47" s="1">
+        <v>0</v>
+      </c>
+      <c r="G47" s="1">
+        <v>0</v>
+      </c>
+      <c r="H47" s="1">
+        <v>0</v>
+      </c>
+      <c r="I47" s="1">
+        <v>0</v>
+      </c>
+      <c r="J47" s="1">
+        <v>0</v>
+      </c>
+      <c r="K47" s="1">
+        <v>0</v>
+      </c>
+      <c r="L47" s="1">
+        <v>0</v>
+      </c>
+      <c r="M47" s="1">
+        <v>0</v>
+      </c>
+      <c r="N47" s="1">
+        <v>0</v>
+      </c>
+      <c r="O47" s="1">
+        <v>0</v>
+      </c>
+      <c r="P47" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q47" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>0</v>
       </c>
@@ -1231,8 +2943,44 @@
       <c r="E48">
         <v>0</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F48" s="1">
+        <v>0</v>
+      </c>
+      <c r="G48" s="1">
+        <v>0</v>
+      </c>
+      <c r="H48" s="1">
+        <v>0</v>
+      </c>
+      <c r="I48" s="1">
+        <v>0</v>
+      </c>
+      <c r="J48" s="1">
+        <v>0</v>
+      </c>
+      <c r="K48" s="1">
+        <v>0</v>
+      </c>
+      <c r="L48" s="1">
+        <v>0</v>
+      </c>
+      <c r="M48" s="1">
+        <v>0</v>
+      </c>
+      <c r="N48" s="1">
+        <v>0</v>
+      </c>
+      <c r="O48" s="1">
+        <v>0</v>
+      </c>
+      <c r="P48" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q48" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>0</v>
       </c>
@@ -1248,8 +2996,44 @@
       <c r="E49">
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F49" s="1">
+        <v>0</v>
+      </c>
+      <c r="G49" s="1">
+        <v>0</v>
+      </c>
+      <c r="H49" s="1">
+        <v>0</v>
+      </c>
+      <c r="I49" s="1">
+        <v>0</v>
+      </c>
+      <c r="J49" s="1">
+        <v>0</v>
+      </c>
+      <c r="K49" s="1">
+        <v>0</v>
+      </c>
+      <c r="L49" s="1">
+        <v>0</v>
+      </c>
+      <c r="M49" s="1">
+        <v>0</v>
+      </c>
+      <c r="N49" s="1">
+        <v>0</v>
+      </c>
+      <c r="O49" s="1">
+        <v>0</v>
+      </c>
+      <c r="P49" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q49" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>0</v>
       </c>
@@ -1265,8 +3049,44 @@
       <c r="E50">
         <v>0</v>
       </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F50" s="1">
+        <v>0</v>
+      </c>
+      <c r="G50" s="1">
+        <v>0</v>
+      </c>
+      <c r="H50" s="1">
+        <v>0</v>
+      </c>
+      <c r="I50" s="1">
+        <v>0</v>
+      </c>
+      <c r="J50" s="1">
+        <v>0</v>
+      </c>
+      <c r="K50" s="1">
+        <v>0</v>
+      </c>
+      <c r="L50" s="1">
+        <v>0</v>
+      </c>
+      <c r="M50" s="1">
+        <v>0</v>
+      </c>
+      <c r="N50" s="1">
+        <v>0</v>
+      </c>
+      <c r="O50" s="1">
+        <v>0</v>
+      </c>
+      <c r="P50" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q50" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>0</v>
       </c>
@@ -1282,8 +3102,44 @@
       <c r="E51">
         <v>296</v>
       </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F51" s="1">
+        <v>304</v>
+      </c>
+      <c r="G51" s="1">
+        <v>0</v>
+      </c>
+      <c r="H51" s="1">
+        <v>0</v>
+      </c>
+      <c r="I51" s="1">
+        <v>0</v>
+      </c>
+      <c r="J51" s="1">
+        <v>0</v>
+      </c>
+      <c r="K51" s="1">
+        <v>0</v>
+      </c>
+      <c r="L51" s="1">
+        <v>0</v>
+      </c>
+      <c r="M51" s="1">
+        <v>0</v>
+      </c>
+      <c r="N51" s="1">
+        <v>0</v>
+      </c>
+      <c r="O51" s="1">
+        <v>0</v>
+      </c>
+      <c r="P51" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q51" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>0</v>
       </c>
@@ -1299,8 +3155,44 @@
       <c r="E52">
         <v>280</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F52" s="1">
+        <v>288</v>
+      </c>
+      <c r="G52" s="1">
+        <v>0</v>
+      </c>
+      <c r="H52" s="1">
+        <v>0</v>
+      </c>
+      <c r="I52" s="1">
+        <v>0</v>
+      </c>
+      <c r="J52" s="1">
+        <v>0</v>
+      </c>
+      <c r="K52" s="1">
+        <v>0</v>
+      </c>
+      <c r="L52" s="1">
+        <v>0</v>
+      </c>
+      <c r="M52" s="1">
+        <v>0</v>
+      </c>
+      <c r="N52" s="1">
+        <v>0</v>
+      </c>
+      <c r="O52" s="1">
+        <v>0</v>
+      </c>
+      <c r="P52" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q52" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>0</v>
       </c>
@@ -1316,8 +3208,44 @@
       <c r="E53">
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F53" s="1">
+        <v>0</v>
+      </c>
+      <c r="G53" s="1">
+        <v>0</v>
+      </c>
+      <c r="H53" s="1">
+        <v>0</v>
+      </c>
+      <c r="I53" s="1">
+        <v>0</v>
+      </c>
+      <c r="J53" s="1">
+        <v>0</v>
+      </c>
+      <c r="K53" s="1">
+        <v>0</v>
+      </c>
+      <c r="L53" s="1">
+        <v>0</v>
+      </c>
+      <c r="M53" s="1">
+        <v>0</v>
+      </c>
+      <c r="N53" s="1">
+        <v>0</v>
+      </c>
+      <c r="O53" s="1">
+        <v>0</v>
+      </c>
+      <c r="P53" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q53" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>0</v>
       </c>
@@ -1333,8 +3261,44 @@
       <c r="E54">
         <v>0</v>
       </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F54" s="1">
+        <v>0</v>
+      </c>
+      <c r="G54" s="1">
+        <v>0</v>
+      </c>
+      <c r="H54" s="1">
+        <v>0</v>
+      </c>
+      <c r="I54" s="1">
+        <v>0</v>
+      </c>
+      <c r="J54" s="1">
+        <v>0</v>
+      </c>
+      <c r="K54" s="1">
+        <v>0</v>
+      </c>
+      <c r="L54" s="1">
+        <v>0</v>
+      </c>
+      <c r="M54" s="1">
+        <v>0</v>
+      </c>
+      <c r="N54" s="1">
+        <v>0</v>
+      </c>
+      <c r="O54" s="1">
+        <v>0</v>
+      </c>
+      <c r="P54" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q54" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>0</v>
       </c>
@@ -1350,8 +3314,44 @@
       <c r="E55">
         <v>16</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F55" s="1">
+        <v>16</v>
+      </c>
+      <c r="G55" s="1">
+        <v>8</v>
+      </c>
+      <c r="H55" s="1">
+        <v>16</v>
+      </c>
+      <c r="I55" s="1">
+        <v>16</v>
+      </c>
+      <c r="J55" s="1">
+        <v>-16</v>
+      </c>
+      <c r="K55" s="1">
+        <v>16</v>
+      </c>
+      <c r="L55" s="1">
+        <v>8</v>
+      </c>
+      <c r="M55" s="1">
+        <v>8</v>
+      </c>
+      <c r="N55" s="1">
+        <v>8</v>
+      </c>
+      <c r="O55" s="1">
+        <v>8</v>
+      </c>
+      <c r="P55" s="1">
+        <v>8</v>
+      </c>
+      <c r="Q55" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>0</v>
       </c>
@@ -1367,8 +3367,44 @@
       <c r="E56">
         <v>8</v>
       </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F56" s="1">
+        <v>16</v>
+      </c>
+      <c r="G56" s="1">
+        <v>8</v>
+      </c>
+      <c r="H56" s="1">
+        <v>8</v>
+      </c>
+      <c r="I56" s="1">
+        <v>8</v>
+      </c>
+      <c r="J56" s="1">
+        <v>0</v>
+      </c>
+      <c r="K56" s="1">
+        <v>8</v>
+      </c>
+      <c r="L56" s="1">
+        <v>0</v>
+      </c>
+      <c r="M56" s="1">
+        <v>0</v>
+      </c>
+      <c r="N56" s="1">
+        <v>0</v>
+      </c>
+      <c r="O56" s="1">
+        <v>8</v>
+      </c>
+      <c r="P56" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>0</v>
       </c>
@@ -1384,8 +3420,44 @@
       <c r="E57">
         <v>56</v>
       </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F57" s="1">
+        <v>64</v>
+      </c>
+      <c r="G57" s="1">
+        <v>56</v>
+      </c>
+      <c r="H57" s="1">
+        <v>64</v>
+      </c>
+      <c r="I57" s="1">
+        <v>64</v>
+      </c>
+      <c r="J57" s="1">
+        <v>56</v>
+      </c>
+      <c r="K57" s="1">
+        <v>64</v>
+      </c>
+      <c r="L57" s="1">
+        <v>64</v>
+      </c>
+      <c r="M57" s="1">
+        <v>56</v>
+      </c>
+      <c r="N57" s="1">
+        <v>56</v>
+      </c>
+      <c r="O57" s="1">
+        <v>56</v>
+      </c>
+      <c r="P57" s="1">
+        <v>56</v>
+      </c>
+      <c r="Q57" s="1">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>0</v>
       </c>
@@ -1401,8 +3473,44 @@
       <c r="E58">
         <v>80</v>
       </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F58" s="1">
+        <v>80</v>
+      </c>
+      <c r="G58" s="1">
+        <v>80</v>
+      </c>
+      <c r="H58" s="1">
+        <v>80</v>
+      </c>
+      <c r="I58" s="1">
+        <v>80</v>
+      </c>
+      <c r="J58" s="1">
+        <v>80</v>
+      </c>
+      <c r="K58" s="1">
+        <v>80</v>
+      </c>
+      <c r="L58" s="1">
+        <v>72</v>
+      </c>
+      <c r="M58" s="1">
+        <v>80</v>
+      </c>
+      <c r="N58" s="1">
+        <v>80</v>
+      </c>
+      <c r="O58" s="1">
+        <v>80</v>
+      </c>
+      <c r="P58" s="1">
+        <v>80</v>
+      </c>
+      <c r="Q58" s="1">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>0</v>
       </c>
@@ -1418,8 +3526,44 @@
       <c r="E59">
         <v>0</v>
       </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F59" s="1">
+        <v>8</v>
+      </c>
+      <c r="G59" s="1">
+        <v>0</v>
+      </c>
+      <c r="H59" s="1">
+        <v>8</v>
+      </c>
+      <c r="I59" s="1">
+        <v>8</v>
+      </c>
+      <c r="J59" s="1">
+        <v>0</v>
+      </c>
+      <c r="K59" s="1">
+        <v>8</v>
+      </c>
+      <c r="L59" s="1">
+        <v>0</v>
+      </c>
+      <c r="M59" s="1">
+        <v>0</v>
+      </c>
+      <c r="N59" s="1">
+        <v>-0</v>
+      </c>
+      <c r="O59" s="1">
+        <v>0</v>
+      </c>
+      <c r="P59" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q59" s="1">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>0</v>
       </c>
@@ -1435,8 +3579,44 @@
       <c r="E60">
         <v>72</v>
       </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F60" s="1">
+        <v>80</v>
+      </c>
+      <c r="G60" s="1">
+        <v>72</v>
+      </c>
+      <c r="H60" s="1">
+        <v>80</v>
+      </c>
+      <c r="I60" s="1">
+        <v>80</v>
+      </c>
+      <c r="J60" s="1">
+        <v>64</v>
+      </c>
+      <c r="K60" s="1">
+        <v>72</v>
+      </c>
+      <c r="L60" s="1">
+        <v>72</v>
+      </c>
+      <c r="M60" s="1">
+        <v>72</v>
+      </c>
+      <c r="N60" s="1">
+        <v>72</v>
+      </c>
+      <c r="O60" s="1">
+        <v>72</v>
+      </c>
+      <c r="P60" s="1">
+        <v>72</v>
+      </c>
+      <c r="Q60" s="1">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>0</v>
       </c>
@@ -1452,8 +3632,44 @@
       <c r="E61">
         <v>0</v>
       </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F61" s="1">
+        <v>0</v>
+      </c>
+      <c r="G61" s="1">
+        <v>0</v>
+      </c>
+      <c r="H61" s="1">
+        <v>0</v>
+      </c>
+      <c r="I61" s="1">
+        <v>0</v>
+      </c>
+      <c r="J61" s="1">
+        <v>0</v>
+      </c>
+      <c r="K61" s="1">
+        <v>0</v>
+      </c>
+      <c r="L61" s="1">
+        <v>0</v>
+      </c>
+      <c r="M61" s="1">
+        <v>0</v>
+      </c>
+      <c r="N61" s="1">
+        <v>0</v>
+      </c>
+      <c r="O61" s="1">
+        <v>0</v>
+      </c>
+      <c r="P61" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q61" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>0</v>
       </c>
@@ -1469,8 +3685,44 @@
       <c r="E62">
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F62" s="1">
+        <v>0</v>
+      </c>
+      <c r="G62" s="1">
+        <v>0</v>
+      </c>
+      <c r="H62" s="1">
+        <v>0</v>
+      </c>
+      <c r="I62" s="1">
+        <v>0</v>
+      </c>
+      <c r="J62" s="1">
+        <v>0</v>
+      </c>
+      <c r="K62" s="1">
+        <v>0</v>
+      </c>
+      <c r="L62" s="1">
+        <v>0</v>
+      </c>
+      <c r="M62" s="1">
+        <v>0</v>
+      </c>
+      <c r="N62" s="1">
+        <v>0</v>
+      </c>
+      <c r="O62" s="1">
+        <v>0</v>
+      </c>
+      <c r="P62" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q62" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>0</v>
       </c>
@@ -1486,8 +3738,44 @@
       <c r="E63">
         <v>0</v>
       </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F63" s="1">
+        <v>0</v>
+      </c>
+      <c r="G63" s="1">
+        <v>0</v>
+      </c>
+      <c r="H63" s="1">
+        <v>0</v>
+      </c>
+      <c r="I63" s="1">
+        <v>0</v>
+      </c>
+      <c r="J63" s="1">
+        <v>0</v>
+      </c>
+      <c r="K63" s="1">
+        <v>0</v>
+      </c>
+      <c r="L63" s="1">
+        <v>0</v>
+      </c>
+      <c r="M63" s="1">
+        <v>0</v>
+      </c>
+      <c r="N63" s="1">
+        <v>0</v>
+      </c>
+      <c r="O63" s="1">
+        <v>0</v>
+      </c>
+      <c r="P63" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q63" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>0</v>
       </c>
@@ -1503,8 +3791,44 @@
       <c r="E64">
         <v>0</v>
       </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F64" s="1">
+        <v>0</v>
+      </c>
+      <c r="G64" s="1">
+        <v>0</v>
+      </c>
+      <c r="H64" s="1">
+        <v>0</v>
+      </c>
+      <c r="I64" s="1">
+        <v>0</v>
+      </c>
+      <c r="J64" s="1">
+        <v>0</v>
+      </c>
+      <c r="K64" s="1">
+        <v>0</v>
+      </c>
+      <c r="L64" s="1">
+        <v>0</v>
+      </c>
+      <c r="M64" s="1">
+        <v>0</v>
+      </c>
+      <c r="N64" s="1">
+        <v>0</v>
+      </c>
+      <c r="O64" s="1">
+        <v>0</v>
+      </c>
+      <c r="P64" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q64" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>0</v>
       </c>
@@ -1520,8 +3844,44 @@
       <c r="E65">
         <v>0</v>
       </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F65" s="1">
+        <v>0</v>
+      </c>
+      <c r="G65" s="1">
+        <v>0</v>
+      </c>
+      <c r="H65" s="1">
+        <v>0</v>
+      </c>
+      <c r="I65" s="1">
+        <v>0</v>
+      </c>
+      <c r="J65" s="1">
+        <v>0</v>
+      </c>
+      <c r="K65" s="1">
+        <v>0</v>
+      </c>
+      <c r="L65" s="1">
+        <v>0</v>
+      </c>
+      <c r="M65" s="1">
+        <v>0</v>
+      </c>
+      <c r="N65" s="1">
+        <v>0</v>
+      </c>
+      <c r="O65" s="1">
+        <v>0</v>
+      </c>
+      <c r="P65" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q65" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>0</v>
       </c>
@@ -1537,8 +3897,44 @@
       <c r="E66">
         <v>0</v>
       </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F66" s="1">
+        <v>0</v>
+      </c>
+      <c r="G66" s="1">
+        <v>0</v>
+      </c>
+      <c r="H66" s="1">
+        <v>0</v>
+      </c>
+      <c r="I66" s="1">
+        <v>0</v>
+      </c>
+      <c r="J66" s="1">
+        <v>0</v>
+      </c>
+      <c r="K66" s="1">
+        <v>0</v>
+      </c>
+      <c r="L66" s="1">
+        <v>0</v>
+      </c>
+      <c r="M66" s="1">
+        <v>0</v>
+      </c>
+      <c r="N66" s="1">
+        <v>0</v>
+      </c>
+      <c r="O66" s="1">
+        <v>0</v>
+      </c>
+      <c r="P66" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q66" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>0</v>
       </c>
@@ -1554,8 +3950,44 @@
       <c r="E67">
         <v>0</v>
       </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F67" s="1">
+        <v>0</v>
+      </c>
+      <c r="G67" s="1">
+        <v>0</v>
+      </c>
+      <c r="H67" s="1">
+        <v>0</v>
+      </c>
+      <c r="I67" s="1">
+        <v>0</v>
+      </c>
+      <c r="J67" s="1">
+        <v>0</v>
+      </c>
+      <c r="K67" s="1">
+        <v>0</v>
+      </c>
+      <c r="L67" s="1">
+        <v>0</v>
+      </c>
+      <c r="M67" s="1">
+        <v>0</v>
+      </c>
+      <c r="N67" s="1">
+        <v>0</v>
+      </c>
+      <c r="O67" s="1">
+        <v>0</v>
+      </c>
+      <c r="P67" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q67" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>0</v>
       </c>
@@ -1571,8 +4003,44 @@
       <c r="E68">
         <v>0</v>
       </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F68" s="1">
+        <v>0</v>
+      </c>
+      <c r="G68" s="1">
+        <v>0</v>
+      </c>
+      <c r="H68" s="1">
+        <v>0</v>
+      </c>
+      <c r="I68" s="1">
+        <v>0</v>
+      </c>
+      <c r="J68" s="1">
+        <v>0</v>
+      </c>
+      <c r="K68" s="1">
+        <v>0</v>
+      </c>
+      <c r="L68" s="1">
+        <v>0</v>
+      </c>
+      <c r="M68" s="1">
+        <v>0</v>
+      </c>
+      <c r="N68" s="1">
+        <v>0</v>
+      </c>
+      <c r="O68" s="1">
+        <v>0</v>
+      </c>
+      <c r="P68" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q68" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>0</v>
       </c>
@@ -1588,8 +4056,44 @@
       <c r="E69">
         <v>0</v>
       </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F69" s="1">
+        <v>0</v>
+      </c>
+      <c r="G69" s="1">
+        <v>0</v>
+      </c>
+      <c r="H69" s="1">
+        <v>0</v>
+      </c>
+      <c r="I69" s="1">
+        <v>0</v>
+      </c>
+      <c r="J69" s="1">
+        <v>0</v>
+      </c>
+      <c r="K69" s="1">
+        <v>0</v>
+      </c>
+      <c r="L69" s="1">
+        <v>0</v>
+      </c>
+      <c r="M69" s="1">
+        <v>0</v>
+      </c>
+      <c r="N69" s="1">
+        <v>0</v>
+      </c>
+      <c r="O69" s="1">
+        <v>0</v>
+      </c>
+      <c r="P69" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q69" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>0</v>
       </c>
@@ -1605,8 +4109,44 @@
       <c r="E70">
         <v>0</v>
       </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F70" s="1">
+        <v>0</v>
+      </c>
+      <c r="G70" s="1">
+        <v>0</v>
+      </c>
+      <c r="H70" s="1">
+        <v>0</v>
+      </c>
+      <c r="I70" s="1">
+        <v>0</v>
+      </c>
+      <c r="J70" s="1">
+        <v>0</v>
+      </c>
+      <c r="K70" s="1">
+        <v>0</v>
+      </c>
+      <c r="L70" s="1">
+        <v>0</v>
+      </c>
+      <c r="M70" s="1">
+        <v>0</v>
+      </c>
+      <c r="N70" s="1">
+        <v>0</v>
+      </c>
+      <c r="O70" s="1">
+        <v>0</v>
+      </c>
+      <c r="P70" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q70" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>0</v>
       </c>
@@ -1622,8 +4162,44 @@
       <c r="E71">
         <v>0</v>
       </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F71" s="1">
+        <v>0</v>
+      </c>
+      <c r="G71" s="1">
+        <v>0</v>
+      </c>
+      <c r="H71" s="1">
+        <v>0</v>
+      </c>
+      <c r="I71" s="1">
+        <v>0</v>
+      </c>
+      <c r="J71" s="1">
+        <v>0</v>
+      </c>
+      <c r="K71" s="1">
+        <v>0</v>
+      </c>
+      <c r="L71" s="1">
+        <v>0</v>
+      </c>
+      <c r="M71" s="1">
+        <v>0</v>
+      </c>
+      <c r="N71" s="1">
+        <v>0</v>
+      </c>
+      <c r="O71" s="1">
+        <v>0</v>
+      </c>
+      <c r="P71" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q71" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>0</v>
       </c>
@@ -1639,8 +4215,44 @@
       <c r="E72">
         <v>0</v>
       </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F72" s="1">
+        <v>0</v>
+      </c>
+      <c r="G72" s="1">
+        <v>0</v>
+      </c>
+      <c r="H72" s="1">
+        <v>0</v>
+      </c>
+      <c r="I72" s="1">
+        <v>0</v>
+      </c>
+      <c r="J72" s="1">
+        <v>0</v>
+      </c>
+      <c r="K72" s="1">
+        <v>0</v>
+      </c>
+      <c r="L72" s="1">
+        <v>0</v>
+      </c>
+      <c r="M72" s="1">
+        <v>0</v>
+      </c>
+      <c r="N72" s="1">
+        <v>0</v>
+      </c>
+      <c r="O72" s="1">
+        <v>0</v>
+      </c>
+      <c r="P72" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q72" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>0</v>
       </c>
@@ -1656,8 +4268,44 @@
       <c r="E73">
         <v>0</v>
       </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F73" s="1">
+        <v>0</v>
+      </c>
+      <c r="G73" s="1">
+        <v>0</v>
+      </c>
+      <c r="H73" s="1">
+        <v>0</v>
+      </c>
+      <c r="I73" s="1">
+        <v>0</v>
+      </c>
+      <c r="J73" s="1">
+        <v>0</v>
+      </c>
+      <c r="K73" s="1">
+        <v>0</v>
+      </c>
+      <c r="L73" s="1">
+        <v>0</v>
+      </c>
+      <c r="M73" s="1">
+        <v>0</v>
+      </c>
+      <c r="N73" s="1">
+        <v>0</v>
+      </c>
+      <c r="O73" s="1">
+        <v>0</v>
+      </c>
+      <c r="P73" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q73" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>0</v>
       </c>
@@ -1673,8 +4321,44 @@
       <c r="E74">
         <v>0</v>
       </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F74" s="1">
+        <v>0</v>
+      </c>
+      <c r="G74" s="1">
+        <v>0</v>
+      </c>
+      <c r="H74" s="1">
+        <v>0</v>
+      </c>
+      <c r="I74" s="1">
+        <v>0</v>
+      </c>
+      <c r="J74" s="1">
+        <v>0</v>
+      </c>
+      <c r="K74" s="1">
+        <v>0</v>
+      </c>
+      <c r="L74" s="1">
+        <v>0</v>
+      </c>
+      <c r="M74" s="1">
+        <v>0</v>
+      </c>
+      <c r="N74" s="1">
+        <v>0</v>
+      </c>
+      <c r="O74" s="1">
+        <v>0</v>
+      </c>
+      <c r="P74" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q74" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
         <v>0</v>
       </c>
@@ -1690,8 +4374,44 @@
       <c r="E75">
         <v>0</v>
       </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F75" s="1">
+        <v>0</v>
+      </c>
+      <c r="G75" s="1">
+        <v>0</v>
+      </c>
+      <c r="H75" s="1">
+        <v>0</v>
+      </c>
+      <c r="I75" s="1">
+        <v>0</v>
+      </c>
+      <c r="J75" s="1">
+        <v>0</v>
+      </c>
+      <c r="K75" s="1">
+        <v>0</v>
+      </c>
+      <c r="L75" s="1">
+        <v>0</v>
+      </c>
+      <c r="M75" s="1">
+        <v>0</v>
+      </c>
+      <c r="N75" s="1">
+        <v>0</v>
+      </c>
+      <c r="O75" s="1">
+        <v>0</v>
+      </c>
+      <c r="P75" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q75" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
         <v>0</v>
       </c>
@@ -1707,8 +4427,44 @@
       <c r="E76">
         <v>0</v>
       </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F76" s="1">
+        <v>0</v>
+      </c>
+      <c r="G76" s="1">
+        <v>0</v>
+      </c>
+      <c r="H76" s="1">
+        <v>0</v>
+      </c>
+      <c r="I76" s="1">
+        <v>0</v>
+      </c>
+      <c r="J76" s="1">
+        <v>0</v>
+      </c>
+      <c r="K76" s="1">
+        <v>0</v>
+      </c>
+      <c r="L76" s="1">
+        <v>0</v>
+      </c>
+      <c r="M76" s="1">
+        <v>0</v>
+      </c>
+      <c r="N76" s="1">
+        <v>0</v>
+      </c>
+      <c r="O76" s="1">
+        <v>0</v>
+      </c>
+      <c r="P76" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q76" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>0</v>
       </c>
@@ -1724,8 +4480,44 @@
       <c r="E77">
         <v>0</v>
       </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F77" s="1">
+        <v>0</v>
+      </c>
+      <c r="G77" s="1">
+        <v>0</v>
+      </c>
+      <c r="H77" s="1">
+        <v>0</v>
+      </c>
+      <c r="I77" s="1">
+        <v>0</v>
+      </c>
+      <c r="J77" s="1">
+        <v>0</v>
+      </c>
+      <c r="K77" s="1">
+        <v>0</v>
+      </c>
+      <c r="L77" s="1">
+        <v>0</v>
+      </c>
+      <c r="M77" s="1">
+        <v>0</v>
+      </c>
+      <c r="N77" s="1">
+        <v>0</v>
+      </c>
+      <c r="O77" s="1">
+        <v>0</v>
+      </c>
+      <c r="P77" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q77" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
         <v>0</v>
       </c>
@@ -1741,8 +4533,44 @@
       <c r="E78">
         <v>0</v>
       </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F78" s="1">
+        <v>0</v>
+      </c>
+      <c r="G78" s="1">
+        <v>0</v>
+      </c>
+      <c r="H78" s="1">
+        <v>0</v>
+      </c>
+      <c r="I78" s="1">
+        <v>0</v>
+      </c>
+      <c r="J78" s="1">
+        <v>0</v>
+      </c>
+      <c r="K78" s="1">
+        <v>0</v>
+      </c>
+      <c r="L78" s="1">
+        <v>0</v>
+      </c>
+      <c r="M78" s="1">
+        <v>0</v>
+      </c>
+      <c r="N78" s="1">
+        <v>0</v>
+      </c>
+      <c r="O78" s="1">
+        <v>0</v>
+      </c>
+      <c r="P78" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q78" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
         <v>0</v>
       </c>
@@ -1758,8 +4586,44 @@
       <c r="E79">
         <v>0</v>
       </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F79" s="1">
+        <v>0</v>
+      </c>
+      <c r="G79" s="1">
+        <v>0</v>
+      </c>
+      <c r="H79" s="1">
+        <v>0</v>
+      </c>
+      <c r="I79" s="1">
+        <v>0</v>
+      </c>
+      <c r="J79" s="1">
+        <v>0</v>
+      </c>
+      <c r="K79" s="1">
+        <v>0</v>
+      </c>
+      <c r="L79" s="1">
+        <v>0</v>
+      </c>
+      <c r="M79" s="1">
+        <v>0</v>
+      </c>
+      <c r="N79" s="1">
+        <v>0</v>
+      </c>
+      <c r="O79" s="1">
+        <v>0</v>
+      </c>
+      <c r="P79" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q79" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
         <v>0</v>
       </c>
@@ -1773,6 +4637,42 @@
         <v>0</v>
       </c>
       <c r="E80">
+        <v>0</v>
+      </c>
+      <c r="F80" s="1">
+        <v>0</v>
+      </c>
+      <c r="G80" s="1">
+        <v>0</v>
+      </c>
+      <c r="H80" s="1">
+        <v>0</v>
+      </c>
+      <c r="I80" s="1">
+        <v>0</v>
+      </c>
+      <c r="J80" s="1">
+        <v>0</v>
+      </c>
+      <c r="K80" s="1">
+        <v>0</v>
+      </c>
+      <c r="L80" s="1">
+        <v>0</v>
+      </c>
+      <c r="M80" s="1">
+        <v>0</v>
+      </c>
+      <c r="N80" s="1">
+        <v>0</v>
+      </c>
+      <c r="O80" s="1">
+        <v>0</v>
+      </c>
+      <c r="P80" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q80" s="1">
         <v>0</v>
       </c>
     </row>

</xml_diff>